<commit_message>
feat: add CEN Deliverables sheet to control panel, fix stale milestones
Sheet 7 tracks all 4 phases of CEN partnership deliverables:
- Phase overview (4 phases, status + packaging gap highlighted)
- Phase 1 deliverables (4 items — work done, folder empty)
- Phase 2 deliverables (7 items — evidence package exists, folder empty)
- Phase 3 deliverables (4 items — validation meeting ~April 17, CRITICAL)
- Phase 4 deliverables (3 items — May, final report)
- CEN input materials inventory (13 documents received)

Also corrected Dashboard and Thesis Evidence sheets:
- CEN Phase 2 marked DONE (completed session 25, Apr 7)
- Next milestone updated to Phase 3 validation ~April 17

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROL_PANEL.xlsx
+++ b/CONTROL_PANEL.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis Evidence" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebase Inventory" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CEN Deliverables" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0 &quot;days&quot;"/>
     <numFmt numFmtId="165" formatCode="0 &quot;of 15&quot;"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,8 +109,56 @@
       <color rgb="00263238"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0000838F"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="009E9E9E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0000838F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00263238"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00D32F2F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FF6F00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -164,8 +213,26 @@
         <bgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000838F"/>
+        <bgColor rgb="0000838F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEBEE"/>
+        <bgColor rgb="00FFEBEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000BCD4"/>
+        <bgColor rgb="0000BCD4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -188,11 +255,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BDBDBD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BDBDBD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BDBDBD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -255,6 +336,71 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -689,9 +835,9 @@
           <t>Next Milestone</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>CEN Phase 2 — April 14</t>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Phase 3 validation — ~April 17</t>
         </is>
       </c>
     </row>
@@ -3590,6 +3736,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="16.8" customHeight="1" s="17">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -3997,6 +4144,8 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16" ht="19.2" customHeight="1" s="17">
       <c r="A16" s="16" t="inlineStr">
         <is>
@@ -4024,17 +4173,17 @@
     <row r="18" ht="75" customHeight="1" s="17">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>April 14, 2026</t>
+          <t>April 14 (DONE)</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>CEN Phase 2 scoring deadline</t>
+          <t>CEN Phase 2 scoring — COMPLETE (session 25, Apr 7)</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>BLOCKING — no slip tolerance</t>
+          <t>BSC comparison 5/6. Evidence package ready.</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4813,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="17">
       <c r="A18" s="23" t="inlineStr">
         <is>
@@ -5176,4 +5324,1752 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF6F00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="17" min="1" max="1"/>
+    <col width="35" customWidth="1" style="17" min="2" max="2"/>
+    <col width="14" customWidth="1" style="17" min="3" max="3"/>
+    <col width="16" customWidth="1" style="17" min="4" max="4"/>
+    <col width="22" customWidth="1" style="17" min="5" max="5"/>
+    <col width="38" customWidth="1" style="17" min="6" max="6"/>
+    <col width="12" customWidth="1" style="17" min="7" max="7"/>
+    <col width="45" customWidth="1" style="17" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>CEN PARTNERSHIP — DELIVERABLES TRACKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>External Partner: Coherence Partnership Quannex x CEN  |  Path: Final Thesis/Thesis Work/External Partners/Coherence Partnership Quannex x CEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>PHASE OVERVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>Date Window</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>Work Done?</t>
+        </is>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>Packaged?</t>
+        </is>
+      </c>
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>Delivery Folder</t>
+        </is>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="inlineStr">
+        <is>
+          <t>Kick-off + interview + synthesis</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Mar 9-20</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F6" s="40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables from Quannex/Phase 1</t>
+        </is>
+      </c>
+      <c r="H6" s="36" t="inlineStr">
+        <is>
+          <t>Interview Mar 20, synthesis complete. FOLDER EMPTY — needs packaging</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>Scoring + BSC comparison + evidence</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>Apr 1-14</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E7" s="39" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables from Quannex/Phase 2</t>
+        </is>
+      </c>
+      <c r="H7" s="36" t="inlineStr">
+        <is>
+          <t>Both questionnaires returned Apr 7. 14-doc evidence package. BSC 5/6. FOLDER EMPTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="inlineStr">
+        <is>
+          <t>Validation session with D + E</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>Apr 15-30</t>
+        </is>
+      </c>
+      <c r="D8" s="42" t="inlineStr">
+        <is>
+          <t>UPCOMING</t>
+        </is>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F8" s="43" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables from Quannex/Phase 3</t>
+        </is>
+      </c>
+      <c r="H8" s="36" t="inlineStr">
+        <is>
+          <t>Present coherence portrait. ~Apr 17. Prepare CEN-facing summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="inlineStr">
+        <is>
+          <t>Final report + recommendations</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="D9" s="43" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G9" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables from Quannex/Phase 4</t>
+        </is>
+      </c>
+      <c r="H9" s="36" t="inlineStr">
+        <is>
+          <t>Depends on Ch5 + cross-case analysis completion</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>PHASE 1 DELIVERABLES — Package into: Deliverables from Quannex/Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="44" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>Source Material</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
+        <is>
+          <t>Source Location</t>
+        </is>
+      </c>
+      <c r="D12" s="44" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="E12" s="44" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F12" s="44" t="inlineStr">
+        <is>
+          <t>Action Needed</t>
+        </is>
+      </c>
+      <c r="G12" s="44" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H12" s="44" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="45" t="inlineStr">
+        <is>
+          <t>Interview Synthesis Report</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Phase1_Interview_Synthesis.md (57 KB)</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase1/</t>
+        </is>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E13" s="46" t="inlineStr">
+        <is>
+          <t>EXISTS — needs formatting</t>
+        </is>
+      </c>
+      <c r="F13" s="36" t="inlineStr">
+        <is>
+          <t>Convert to branded PDF, add exec summary</t>
+        </is>
+      </c>
+      <c r="G13" s="47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H13" s="36" t="inlineStr">
+        <is>
+          <t>Core research artifact — shows CEN their organizational portrait from Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="45" t="inlineStr">
+        <is>
+          <t>Preliminary Face Mapping</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Preliminary_Face_Mapping.md (33 KB)</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase1/</t>
+        </is>
+      </c>
+      <c r="D14" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>EXISTS — needs formatting</t>
+        </is>
+      </c>
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>Convert to branded PDF with visual dodecahedron diagram</t>
+        </is>
+      </c>
+      <c r="G14" s="47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H14" s="36" t="inlineStr">
+        <is>
+          <t>Shows how CEN's domains map to the 12 faces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="45" t="inlineStr">
+        <is>
+          <t>Meeting Transcript</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>20-03-2026_PHASE1_Meeting-TRANSCRIPT.md (183 KB)</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase1/</t>
+        </is>
+      </c>
+      <c r="D15" s="37" t="inlineStr">
+        <is>
+          <t>PDF or MD</t>
+        </is>
+      </c>
+      <c r="E15" s="48" t="inlineStr">
+        <is>
+          <t>EXISTS — decide if CEN-facing</t>
+        </is>
+      </c>
+      <c r="F15" s="36" t="inlineStr">
+        <is>
+          <t>Review for sensitivity, redact if needed</t>
+        </is>
+      </c>
+      <c r="G15" s="49" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="H15" s="36" t="inlineStr">
+        <is>
+          <t>May not need to be delivered — check partnership agreement</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="45" t="inlineStr">
+        <is>
+          <t>Personal Notes</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="inlineStr">
+        <is>
+          <t>Personal Notes - Fresh, right after the meeting!.md</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase1/</t>
+        </is>
+      </c>
+      <c r="D16" s="37" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E16" s="48" t="inlineStr">
+        <is>
+          <t>INTERNAL ONLY</t>
+        </is>
+      </c>
+      <c r="F16" s="36" t="inlineStr">
+        <is>
+          <t>Do NOT deliver — keep as research evidence</t>
+        </is>
+      </c>
+      <c r="G16" s="37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="36" t="inlineStr">
+        <is>
+          <t>Raw observations, thesis evidence only</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>PHASE 2 DELIVERABLES — Package into: Deliverables from Quannex/Phase 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>Source Material</t>
+        </is>
+      </c>
+      <c r="C19" s="44" t="inlineStr">
+        <is>
+          <t>Source Location</t>
+        </is>
+      </c>
+      <c r="D19" s="44" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="E19" s="44" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F19" s="44" t="inlineStr">
+        <is>
+          <t>Action Needed</t>
+        </is>
+      </c>
+      <c r="G19" s="44" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H19" s="44" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="45" t="inlineStr">
+        <is>
+          <t>Coherence Portrait / Vector Diagnostics</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Phase2_C1_VectorDiagnostics.md (20 KB)</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
+        </is>
+      </c>
+      <c r="D20" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E20" s="46" t="inlineStr">
+        <is>
+          <t>EXISTS — needs formatting</t>
+        </is>
+      </c>
+      <c r="F20" s="36" t="inlineStr">
+        <is>
+          <t>Convert to branded CEN-facing report, add visualizations</t>
+        </is>
+      </c>
+      <c r="G20" s="47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H20" s="36" t="inlineStr">
+        <is>
+          <t>The core deliverable — shows CEN their coherence state</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="45" t="inlineStr">
+        <is>
+          <t>Breath Axis Analysis</t>
+        </is>
+      </c>
+      <c r="B21" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Phase2_C2_BreathAxes.md (21 KB)</t>
+        </is>
+      </c>
+      <c r="C21" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
+        </is>
+      </c>
+      <c r="D21" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E21" s="46" t="inlineStr">
+        <is>
+          <t>EXISTS — needs formatting</t>
+        </is>
+      </c>
+      <c r="F21" s="36" t="inlineStr">
+        <is>
+          <t>Format as section of coherence report or standalone</t>
+        </is>
+      </c>
+      <c r="G21" s="47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H21" s="36" t="inlineStr">
+        <is>
+          <t>Polarity tensions — key insight for leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="45" t="inlineStr">
+        <is>
+          <t>Divergence Narratives (Hidden Tensions)</t>
+        </is>
+      </c>
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Phase2_C3_DivergenceNarratives.md (13 KB)</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
+        </is>
+      </c>
+      <c r="D22" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E22" s="46" t="inlineStr">
+        <is>
+          <t>EXISTS — needs formatting</t>
+        </is>
+      </c>
+      <c r="F22" s="36" t="inlineStr">
+        <is>
+          <t>Sensitive content — frame constructively for CEN</t>
+        </is>
+      </c>
+      <c r="G22" s="47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H22" s="36" t="inlineStr">
+        <is>
+          <t>Where co-founders diverge — handle with care</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>BSC Comparison Report</t>
+        </is>
+      </c>
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Phase2_C4_BSCComparison.md (27 KB)</t>
+        </is>
+      </c>
+      <c r="C23" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
+        </is>
+      </c>
+      <c r="D23" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E23" s="46" t="inlineStr">
+        <is>
+          <t>EXISTS — needs formatting</t>
+        </is>
+      </c>
+      <c r="F23" s="36" t="inlineStr">
+        <is>
+          <t>Format as comparison report: Spiral vs BSC (5/6 verdict)</t>
+        </is>
+      </c>
+      <c r="G23" s="47" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H23" s="36" t="inlineStr">
+        <is>
+          <t>Academic evidence + CEN value prop: shows what Spiral adds over BSC</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>Raw Scoring Data (Frozen)</t>
+        </is>
+      </c>
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Phase2_RawScores_Frozen.md (9 KB)</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
+        </is>
+      </c>
+      <c r="D24" s="37" t="inlineStr">
+        <is>
+          <t>PDF or Excel</t>
+        </is>
+      </c>
+      <c r="E24" s="48" t="inlineStr">
+        <is>
+          <t>EXISTS — decide if CEN-facing</t>
+        </is>
+      </c>
+      <c r="F24" s="36" t="inlineStr">
+        <is>
+          <t>May include as appendix to coherence portrait</t>
+        </is>
+      </c>
+      <c r="G24" s="49" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="H24" s="36" t="inlineStr">
+        <is>
+          <t>Both co-founders' scores, independence verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="45" t="inlineStr">
+        <is>
+          <t>Scoring Questionnaires (Completed)</t>
+        </is>
+      </c>
+      <c r="B25" s="36" t="inlineStr">
+        <is>
+          <t>Dominique + Esther completed questionnaires</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/CEN_Scoring_Questionnaire/</t>
+        </is>
+      </c>
+      <c r="D25" s="37" t="inlineStr">
+        <is>
+          <t>DOCX (as-is)</t>
+        </is>
+      </c>
+      <c r="E25" s="50" t="inlineStr">
+        <is>
+          <t>COMPLETE — already received</t>
+        </is>
+      </c>
+      <c r="F25" s="36" t="inlineStr">
+        <is>
+          <t>Archive copies in Phase 2 folder for completeness</t>
+        </is>
+      </c>
+      <c r="G25" s="37" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="H25" s="36" t="inlineStr">
+        <is>
+          <t>Input FROM CEN, not deliverable TO CEN — but archive</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="45" t="inlineStr">
+        <is>
+          <t>Face Guide Companion</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Face_Guide_For_Scoring.pdf (202 KB)</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>Meetings &amp; Planning/CEN_Phase2/</t>
+        </is>
+      </c>
+      <c r="D26" s="37" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E26" s="50" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="F26" s="36" t="inlineStr">
+        <is>
+          <t>Already formatted — copy to Phase 2 folder</t>
+        </is>
+      </c>
+      <c r="G26" s="37" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="H26" s="36" t="inlineStr">
+        <is>
+          <t>Sent to CEN for scoring context</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="inlineStr">
+        <is>
+          <t>PHASE 3 DELIVERABLES — Validation Session (~April 17) — Package into: Deliverables from Quannex/Phase 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="44" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Source Material</t>
+        </is>
+      </c>
+      <c r="C29" s="44" t="inlineStr">
+        <is>
+          <t>Source Location</t>
+        </is>
+      </c>
+      <c r="D29" s="44" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="E29" s="44" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F29" s="44" t="inlineStr">
+        <is>
+          <t>Action Needed</t>
+        </is>
+      </c>
+      <c r="G29" s="44" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H29" s="44" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="45" t="inlineStr">
+        <is>
+          <t>Validation Presentation</t>
+        </is>
+      </c>
+      <c r="B30" s="36" t="inlineStr">
+        <is>
+          <t>To be created from Phase 2 evidence</t>
+        </is>
+      </c>
+      <c r="C30" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D30" s="37" t="inlineStr">
+        <is>
+          <t>PPTX (branded)</t>
+        </is>
+      </c>
+      <c r="E30" s="51" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="F30" s="36" t="inlineStr">
+        <is>
+          <t>Create presentation summarizing coherence portrait + key findings</t>
+        </is>
+      </c>
+      <c r="G30" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="H30" s="36" t="inlineStr">
+        <is>
+          <t>This is what you present to D + E at the validation meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="45" t="inlineStr">
+        <is>
+          <t>CEN-Facing Coherence Summary</t>
+        </is>
+      </c>
+      <c r="B31" s="36" t="inlineStr">
+        <is>
+          <t>Synthesize from C1-C4 evidence docs</t>
+        </is>
+      </c>
+      <c r="C31" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D31" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E31" s="51" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="F31" s="36" t="inlineStr">
+        <is>
+          <t>One-page or two-page executive summary for CEN leadership</t>
+        </is>
+      </c>
+      <c r="G31" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="H31" s="36" t="inlineStr">
+        <is>
+          <t>Leave-behind document after validation session</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="45" t="inlineStr">
+        <is>
+          <t>Validation Session Notes</t>
+        </is>
+      </c>
+      <c r="B32" s="36" t="inlineStr">
+        <is>
+          <t>Will be captured during meeting</t>
+        </is>
+      </c>
+      <c r="C32" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="37" t="inlineStr">
+        <is>
+          <t>MD then PDF</t>
+        </is>
+      </c>
+      <c r="E32" s="48" t="inlineStr">
+        <is>
+          <t>FUTURE</t>
+        </is>
+      </c>
+      <c r="F32" s="36" t="inlineStr">
+        <is>
+          <t>Record CEN's reactions, corrections, confirmations</t>
+        </is>
+      </c>
+      <c r="G32" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H32" s="36" t="inlineStr">
+        <is>
+          <t>Critical thesis evidence — did CEN validate the portrait?</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="45" t="inlineStr">
+        <is>
+          <t>POC Live Demo (optional)</t>
+        </is>
+      </c>
+      <c r="B33" s="36" t="inlineStr">
+        <is>
+          <t>POC codebase — load CEN data into engine</t>
+        </is>
+      </c>
+      <c r="C33" s="41" t="inlineStr">
+        <is>
+          <t>POC/companies/ (needs CEN template)</t>
+        </is>
+      </c>
+      <c r="D33" s="37" t="inlineStr">
+        <is>
+          <t>Live demo</t>
+        </is>
+      </c>
+      <c r="E33" s="48" t="inlineStr">
+        <is>
+          <t>REQUIRES CEN COMPANY TEMPLATE</t>
+        </is>
+      </c>
+      <c r="F33" s="36" t="inlineStr">
+        <is>
+          <t>Create companies/cen/ template from scoring data</t>
+        </is>
+      </c>
+      <c r="G33" s="49" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="H33" s="36" t="inlineStr">
+        <is>
+          <t>Would powerfully demonstrate the tool — consider creating CEN template from Phase 2 scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t>PHASE 4 DELIVERABLES — Final Report (May) — Package into: Deliverables from Quannex/Phase 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="44" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Source Material</t>
+        </is>
+      </c>
+      <c r="C36" s="44" t="inlineStr">
+        <is>
+          <t>Source Location</t>
+        </is>
+      </c>
+      <c r="D36" s="44" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="E36" s="44" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F36" s="44" t="inlineStr">
+        <is>
+          <t>Action Needed</t>
+        </is>
+      </c>
+      <c r="G36" s="44" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H36" s="44" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="45" t="inlineStr">
+        <is>
+          <t>Final Coherence Report</t>
+        </is>
+      </c>
+      <c r="B37" s="36" t="inlineStr">
+        <is>
+          <t>Full synthesis of Phase 1-3 findings</t>
+        </is>
+      </c>
+      <c r="C37" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D37" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E37" s="48" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="F37" s="36" t="inlineStr">
+        <is>
+          <t>Comprehensive CEN coherence assessment with recommendations</t>
+        </is>
+      </c>
+      <c r="G37" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H37" s="36" t="inlineStr">
+        <is>
+          <t>The capstone deliverable — CEN's return on participation</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="45" t="inlineStr">
+        <is>
+          <t>Recommendations Document</t>
+        </is>
+      </c>
+      <c r="B38" s="36" t="inlineStr">
+        <is>
+          <t>Derived from cross-case analysis + validation</t>
+        </is>
+      </c>
+      <c r="C38" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D38" s="37" t="inlineStr">
+        <is>
+          <t>PDF (branded)</t>
+        </is>
+      </c>
+      <c r="E38" s="48" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="F38" s="36" t="inlineStr">
+        <is>
+          <t>Actionable recommendations based on coherence portrait</t>
+        </is>
+      </c>
+      <c r="G38" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H38" s="36" t="inlineStr">
+        <is>
+          <t>Practical value for CEN — not just academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="45" t="inlineStr">
+        <is>
+          <t>Thank You + Next Steps</t>
+        </is>
+      </c>
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C39" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" s="37" t="inlineStr">
+        <is>
+          <t>PDF or letter</t>
+        </is>
+      </c>
+      <c r="E39" s="48" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="F39" s="36" t="inlineStr">
+        <is>
+          <t>Formal closure of research partnership</t>
+        </is>
+      </c>
+      <c r="G39" s="37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="H39" s="36" t="inlineStr">
+        <is>
+          <t>Professional courtesy — partnership confirmation referenced deliverables</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="33" t="inlineStr">
+        <is>
+          <t>CEN INPUT MATERIALS — Documents received from CEN (for reference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="44" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C42" s="44" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="D42" s="44" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="E42" s="44" t="inlineStr">
+        <is>
+          <t>Relevance</t>
+        </is>
+      </c>
+      <c r="F42" s="44" t="inlineStr">
+        <is>
+          <t>Used In</t>
+        </is>
+      </c>
+      <c r="G42" s="44" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H42" s="44" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="36" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="B43" s="45" t="inlineStr">
+        <is>
+          <t>Signed NDA</t>
+        </is>
+      </c>
+      <c r="C43" s="37" t="inlineStr">
+        <is>
+          <t>461 KB</t>
+        </is>
+      </c>
+      <c r="D43" s="41" t="inlineStr">
+        <is>
+          <t>Meeting 1st/</t>
+        </is>
+      </c>
+      <c r="E43" s="37" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F43" s="36" t="inlineStr">
+        <is>
+          <t>All phases</t>
+        </is>
+      </c>
+      <c r="G43" s="36" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="36" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="B44" s="45" t="inlineStr">
+        <is>
+          <t>Signed Partnership Confirmation</t>
+        </is>
+      </c>
+      <c r="C44" s="37" t="inlineStr">
+        <is>
+          <t>409 KB</t>
+        </is>
+      </c>
+      <c r="D44" s="41" t="inlineStr">
+        <is>
+          <t>Meeting 1st/</t>
+        </is>
+      </c>
+      <c r="E44" s="37" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F44" s="36" t="inlineStr">
+        <is>
+          <t>All phases</t>
+        </is>
+      </c>
+      <c r="G44" s="36" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="36" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B45" s="45" t="inlineStr">
+        <is>
+          <t>CEN Business Plan V2.0</t>
+        </is>
+      </c>
+      <c r="C45" s="37" t="inlineStr">
+        <is>
+          <t>~19 MB</t>
+        </is>
+      </c>
+      <c r="D45" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Strategy/</t>
+        </is>
+      </c>
+      <c r="E45" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F45" s="36" t="inlineStr">
+        <is>
+          <t>Phase 1 synthesis</t>
+        </is>
+      </c>
+      <c r="G45" s="36" t="inlineStr">
+        <is>
+          <t>Core strategic context</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="36" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B46" s="45" t="inlineStr">
+        <is>
+          <t>CEN Strategy V0.4</t>
+        </is>
+      </c>
+      <c r="C46" s="37" t="inlineStr">
+        <is>
+          <t>425 KB</t>
+        </is>
+      </c>
+      <c r="D46" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Strategy/</t>
+        </is>
+      </c>
+      <c r="E46" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F46" s="36" t="inlineStr">
+        <is>
+          <t>Phase 1 synthesis</t>
+        </is>
+      </c>
+      <c r="G46" s="36" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="36" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B47" s="45" t="inlineStr">
+        <is>
+          <t>Purpose Vision Mission Values V0.1</t>
+        </is>
+      </c>
+      <c r="C47" s="37" t="inlineStr">
+        <is>
+          <t>25 KB</t>
+        </is>
+      </c>
+      <c r="D47" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Vision Mission/</t>
+        </is>
+      </c>
+      <c r="E47" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F47" s="36" t="inlineStr">
+        <is>
+          <t>Face mapping</t>
+        </is>
+      </c>
+      <c r="G47" s="36" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="36" t="inlineStr">
+        <is>
+          <t>Pillar 1</t>
+        </is>
+      </c>
+      <c r="B48" s="45" t="inlineStr">
+        <is>
+          <t>Conscious Leadership Course Proposal</t>
+        </is>
+      </c>
+      <c r="C48" s="37" t="inlineStr">
+        <is>
+          <t>1.2 MB</t>
+        </is>
+      </c>
+      <c r="D48" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Pillar 1/</t>
+        </is>
+      </c>
+      <c r="E48" s="37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F48" s="36" t="inlineStr">
+        <is>
+          <t>Face 6 (Consciousness)</t>
+        </is>
+      </c>
+      <c r="G48" s="36" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="36" t="inlineStr">
+        <is>
+          <t>Pillar 2</t>
+        </is>
+      </c>
+      <c r="B49" s="45" t="inlineStr">
+        <is>
+          <t>AI Consulting + Governance proposals</t>
+        </is>
+      </c>
+      <c r="C49" s="37" t="inlineStr">
+        <is>
+          <t>~230 KB</t>
+        </is>
+      </c>
+      <c r="D49" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Pillar 2/</t>
+        </is>
+      </c>
+      <c r="E49" s="37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F49" s="36" t="inlineStr">
+        <is>
+          <t>Face 3, Face 11</t>
+        </is>
+      </c>
+      <c r="G49" s="36" t="inlineStr">
+        <is>
+          <t>5 documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="36" t="inlineStr">
+        <is>
+          <t>Pillar 3</t>
+        </is>
+      </c>
+      <c r="B50" s="45" t="inlineStr">
+        <is>
+          <t>LLM, DCS, Business Plans, Partners</t>
+        </is>
+      </c>
+      <c r="C50" s="37" t="inlineStr">
+        <is>
+          <t>~42 MB</t>
+        </is>
+      </c>
+      <c r="D50" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Pillar 3/</t>
+        </is>
+      </c>
+      <c r="E50" s="37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F50" s="36" t="inlineStr">
+        <is>
+          <t>Multiple faces</t>
+        </is>
+      </c>
+      <c r="G50" s="36" t="inlineStr">
+        <is>
+          <t>18 documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="36" t="inlineStr">
+        <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="B51" s="45" t="inlineStr">
+        <is>
+          <t>Volunteer programs + contracts</t>
+        </is>
+      </c>
+      <c r="C51" s="37" t="inlineStr">
+        <is>
+          <t>~470 KB</t>
+        </is>
+      </c>
+      <c r="D51" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Teams/</t>
+        </is>
+      </c>
+      <c r="E51" s="37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F51" s="36" t="inlineStr">
+        <is>
+          <t>Face 4, Face 9</t>
+        </is>
+      </c>
+      <c r="G51" s="36" t="inlineStr">
+        <is>
+          <t>5 documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="36" t="inlineStr">
+        <is>
+          <t>Scoring</t>
+        </is>
+      </c>
+      <c r="B52" s="45" t="inlineStr">
+        <is>
+          <t>Dominique questionnaire (completed)</t>
+        </is>
+      </c>
+      <c r="C52" s="37" t="inlineStr">
+        <is>
+          <t>27 KB</t>
+        </is>
+      </c>
+      <c r="D52" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Scoring/</t>
+        </is>
+      </c>
+      <c r="E52" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="F52" s="36" t="inlineStr">
+        <is>
+          <t>Phase 2 evidence</t>
+        </is>
+      </c>
+      <c r="G52" s="36" t="inlineStr">
+        <is>
+          <t>Returned Apr 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="36" t="inlineStr">
+        <is>
+          <t>Scoring</t>
+        </is>
+      </c>
+      <c r="B53" s="45" t="inlineStr">
+        <is>
+          <t>Esther questionnaire (completed)</t>
+        </is>
+      </c>
+      <c r="C53" s="37" t="inlineStr">
+        <is>
+          <t>30 KB</t>
+        </is>
+      </c>
+      <c r="D53" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Scoring/</t>
+        </is>
+      </c>
+      <c r="E53" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="F53" s="36" t="inlineStr">
+        <is>
+          <t>Phase 2 evidence</t>
+        </is>
+      </c>
+      <c r="G53" s="36" t="inlineStr">
+        <is>
+          <t>Returned Apr 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="36" t="inlineStr">
+        <is>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="B54" s="45" t="inlineStr">
+        <is>
+          <t>Phase 1 Interview (video)</t>
+        </is>
+      </c>
+      <c r="C54" s="37" t="inlineStr">
+        <is>
+          <t>4.08 GB</t>
+        </is>
+      </c>
+      <c r="D54" s="41" t="inlineStr">
+        <is>
+          <t>CEN_Phase1/</t>
+        </is>
+      </c>
+      <c r="E54" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="F54" s="36" t="inlineStr">
+        <is>
+          <t>Phase 1 synthesis</t>
+        </is>
+      </c>
+      <c r="G54" s="36" t="inlineStr">
+        <is>
+          <t>Primary research data</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="36" t="inlineStr">
+        <is>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="B55" s="45" t="inlineStr">
+        <is>
+          <t>Phase 2 Meeting (video)</t>
+        </is>
+      </c>
+      <c r="C55" s="37" t="inlineStr">
+        <is>
+          <t>430 MB</t>
+        </is>
+      </c>
+      <c r="D55" s="41" t="inlineStr">
+        <is>
+          <t>CEN_Phase2/</t>
+        </is>
+      </c>
+      <c r="E55" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="F55" s="36" t="inlineStr">
+        <is>
+          <t>Phase 2 evidence</t>
+        </is>
+      </c>
+      <c r="G55" s="36" t="inlineStr">
+        <is>
+          <t>Primary research data</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="52" t="inlineStr">
+        <is>
+          <t>KEY GAP: Phase 1 and Phase 2 work is DONE but delivery folders are EMPTY. Package existing evidence into branded PDFs before Phase 3 validation (~April 17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="41" t="inlineStr">
+        <is>
+          <t>Folder path: Final Thesis/Thesis Work/External Partners/Coherence Partnership Quannex x CEN/Local Source for CEN facing documents/CEN Facing Folder/Deliverables from Quannex/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="D6:D9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"DONE,UPCOMING,IN PROGRESS,NOT STARTED"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E6:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"YES,NO,PARTIAL"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: rebuild CEN sheet from partnership agreement, add raw scores + packaging actions
Self-critique found 4 promised deliverables missing from the CEN sheet (conventional
analysis, 3D visualization, shadow analysis, proposed KPIs). Rebuilt from the signed
Partnership_Overview_and_FAQ.md as canonical source. New sections:

- 8 promised deliverables with status vs. packaging gap
- 5 phases (added Phase 0 kickoff)
- 8 prioritized packaging actions with effort estimates
- 12 face raw scores from frozen dataset + POC-ready normalized arrays
- 11 CEN input materials inventory
- 4 key gaps identified at bottom

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONTROL_PANEL.xlsx
+++ b/CONTROL_PANEL.xlsx
@@ -232,7 +232,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -269,11 +269,55 @@
         <color rgb="00BDBDBD"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BDBDBD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BDBDBD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BDBDBD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BDBDBD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -402,6 +446,21 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3736,7 +3795,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="16.8" customHeight="1" s="17">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -4144,8 +4202,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16" ht="19.2" customHeight="1" s="17">
       <c r="A16" s="16" t="inlineStr">
         <is>
@@ -5333,15 +5389,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" style="17" min="1" max="1"/>
+    <col width="12" customWidth="1" style="17" min="1" max="1"/>
     <col width="35" customWidth="1" style="17" min="2" max="2"/>
-    <col width="14" customWidth="1" style="17" min="3" max="3"/>
+    <col width="38" customWidth="1" style="17" min="3" max="3"/>
     <col width="16" customWidth="1" style="17" min="4" max="4"/>
-    <col width="22" customWidth="1" style="17" min="5" max="5"/>
-    <col width="38" customWidth="1" style="17" min="6" max="6"/>
+    <col width="35" customWidth="1" style="17" min="5" max="5"/>
+    <col width="14" customWidth="1" style="17" min="6" max="6"/>
     <col width="12" customWidth="1" style="17" min="7" max="7"/>
     <col width="45" customWidth="1" style="17" min="8" max="8"/>
   </cols>
@@ -5349,1727 +5405,1989 @@
     <row r="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>CEN PARTNERSHIP — DELIVERABLES TRACKER</t>
+          <t>CEN PARTNERSHIP -- DELIVERABLES TRACKER</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>External Partner: Coherence Partnership Quannex x CEN  |  Path: Final Thesis/Thesis Work/External Partners/Coherence Partnership Quannex x CEN</t>
+          <t>Source: Partnership_Overview_and_FAQ.md (signed scope)  |  Path: Final Thesis/.../Coherence Partnership Quannex x CEN</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="33" t="inlineStr">
         <is>
-          <t>PHASE OVERVIEW</t>
+          <t>PROMISED DELIVERABLES (from Partnership Overview &amp; FAQ, signed Feb 2026)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
         <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Promised Deliverable</t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>Source Material</t>
+        </is>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>Target Phase</t>
+        </is>
+      </c>
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>Packaged?</t>
+        </is>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="45" t="inlineStr">
+        <is>
+          <t>Conventional strategic analysis</t>
+        </is>
+      </c>
+      <c r="C6" s="36" t="inlineStr">
+        <is>
+          <t>PESTEL, Porter's 5 Forces, McKinsey 7S, SWOT, BSC mapping</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E6" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Conventional_Analysis_Working_Draft.md (77KB) + PESTEL notes + 7S analysis</t>
+        </is>
+      </c>
+      <c r="F6" s="37" t="inlineStr">
+        <is>
+          <t>Phase 1-2</t>
+        </is>
+      </c>
+      <c r="G6" s="40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H6" s="36" t="inlineStr">
+        <is>
+          <t>Working draft exists in _Not yet facing/ folder. Post-interview enriched (session 18). Needs CEN-facing format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="45" t="inlineStr">
+        <is>
+          <t>Novel coherence assessment (Spiral Dashboard)</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="inlineStr">
+        <is>
+          <t>Full coherence portrait using Spiral Dashboard methodology</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E7" s="36" t="inlineStr">
+        <is>
+          <t>Phase 2 Evidence Package (14 docs) — Vector Diagnostics, Breath, Divergence, BSC</t>
+        </is>
+      </c>
+      <c r="F7" s="37" t="inlineStr">
+        <is>
+          <t>Phase 2-3</t>
+        </is>
+      </c>
+      <c r="G7" s="40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H7" s="36" t="inlineStr">
+        <is>
+          <t>Core deliverable. Evidence complete, needs branded report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="45" t="inlineStr">
+        <is>
+          <t>3D visualization of CEN's organizational DNA</t>
+        </is>
+      </c>
+      <c r="C8" s="36" t="inlineStr">
+        <is>
+          <t>Interactive dodecahedron reflecting CEN's patterns</t>
+        </is>
+      </c>
+      <c r="D8" s="40" t="inlineStr">
+        <is>
+          <t>REQUIRES CEN TEMPLATE</t>
+        </is>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>POC codebase + CEN raw scores (normalized arrays ready in RawScores_Frozen.md)</t>
+        </is>
+      </c>
+      <c r="F8" s="37" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="G8" s="37" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H8" s="36" t="inlineStr">
+        <is>
+          <t>Need to create companies/cen/ template from Phase 2 scores. Then POC renders it live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="45" t="inlineStr">
+        <is>
+          <t>Shadow analysis</t>
+        </is>
+      </c>
+      <c r="C9" s="36" t="inlineStr">
+        <is>
+          <t>Hidden tensions, blind spots, dormant strengths</t>
+        </is>
+      </c>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="E9" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Phase2_C3_DivergenceNarratives.md covers divergence. Full shadow analysis needs POC run.</t>
+        </is>
+      </c>
+      <c r="F9" s="37" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="G9" s="40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H9" s="36" t="inlineStr">
+        <is>
+          <t>Divergence narratives done. Full shadow detection requires CEN template in POC engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="45" t="inlineStr">
+        <is>
+          <t>Breath analysis</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="inlineStr">
+        <is>
+          <t>6 polarity axes balance assessment</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Phase2_C2_BreathAxes.md (21KB) + raw axis scores frozen</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>Phase 2-3</t>
+        </is>
+      </c>
+      <c r="G10" s="40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H10" s="36" t="inlineStr">
+        <is>
+          <t>Complete with 4-vector data. Needs formatting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="45" t="inlineStr">
+        <is>
+          <t>Debrief session</t>
+        </is>
+      </c>
+      <c r="C11" s="36" t="inlineStr">
+        <is>
+          <t>Discussing findings, implications, actionable next steps</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>UPCOMING</t>
+        </is>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>Phase 3 validation meeting materials (to be prepared)</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H11" s="36" t="inlineStr">
+        <is>
+          <t>~April 17. Presentation + CEN-facing summary needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="45" t="inlineStr">
+        <is>
+          <t>Proposed KPIs with methodology notes</t>
+        </is>
+      </c>
+      <c r="C12" s="36" t="inlineStr">
+        <is>
+          <t>Tailored KPI suggestions for CEN's context</t>
+        </is>
+      </c>
+      <c r="D12" s="43" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>Will derive from coherence portrait + face mapping + breath analysis</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>Phase 3-4</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H12" s="36" t="inlineStr">
+        <is>
+          <t>Promised deliverable — not yet created. Should emerge from the coherence assessment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="37" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="45" t="inlineStr">
+        <is>
+          <t>Thesis acknowledgment</t>
+        </is>
+      </c>
+      <c r="C13" s="36" t="inlineStr">
+        <is>
+          <t>Named acknowledgment in published thesis</t>
+        </is>
+      </c>
+      <c r="D13" s="43" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="E13" s="36" t="inlineStr">
+        <is>
+          <t>Will be written in thesis Chapter 1 or Acknowledgments section</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="G13" s="37" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H13" s="36" t="inlineStr">
+        <is>
+          <t>Write during final thesis assembly (May).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>PHASE OVERVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="B16" s="44" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="C5" s="34" t="inlineStr">
+      <c r="C16" s="44" t="inlineStr">
         <is>
           <t>Date Window</t>
         </is>
       </c>
-      <c r="D5" s="34" t="inlineStr">
+      <c r="D16" s="44" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E5" s="34" t="inlineStr">
+      <c r="E16" s="44" t="inlineStr">
         <is>
           <t>Work Done?</t>
         </is>
       </c>
-      <c r="F5" s="34" t="inlineStr">
+      <c r="F16" s="44" t="inlineStr">
         <is>
           <t>Packaged?</t>
         </is>
       </c>
-      <c r="G5" s="34" t="inlineStr">
+      <c r="G16" s="44" t="inlineStr">
         <is>
           <t>Delivery Folder</t>
         </is>
       </c>
-      <c r="H5" s="34" t="inlineStr">
+      <c r="H16" s="44" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="35" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="B17" s="36" t="inlineStr">
+        <is>
+          <t>Kickoff &amp; orientation</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>Late Feb</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E17" s="39" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F17" s="37" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G17" s="41" t="inlineStr">
+        <is>
+          <t>N/A (meeting only)</t>
+        </is>
+      </c>
+      <c r="H17" s="36" t="inlineStr">
+        <is>
+          <t>Feb 13 meeting. Signed NDA + Partnership. 3D demo shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="B6" s="36" t="inlineStr">
-        <is>
-          <t>Kick-off + interview + synthesis</t>
-        </is>
-      </c>
-      <c r="C6" s="37" t="inlineStr">
-        <is>
-          <t>Mar 9-20</t>
-        </is>
-      </c>
-      <c r="D6" s="38" t="inlineStr">
+      <c r="B18" s="36" t="inlineStr">
+        <is>
+          <t>Conventional analysis + interview</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>Mar 9-31</t>
+        </is>
+      </c>
+      <c r="D18" s="38" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="E6" s="39" t="inlineStr">
+      <c r="E18" s="39" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F6" s="40" t="inlineStr">
+      <c r="F18" s="40" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="G6" s="41" t="inlineStr">
+      <c r="G18" s="41" t="inlineStr">
         <is>
           <t>Deliverables from Quannex/Phase 1</t>
         </is>
       </c>
-      <c r="H6" s="36" t="inlineStr">
-        <is>
-          <t>Interview Mar 20, synthesis complete. FOLDER EMPTY — needs packaging</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="35" t="inlineStr">
+      <c r="H18" s="36" t="inlineStr">
+        <is>
+          <t>Interview Mar 20, synthesis 57KB. FOLDER EMPTY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B7" s="36" t="inlineStr">
+      <c r="B19" s="36" t="inlineStr">
         <is>
           <t>Scoring + BSC comparison + evidence</t>
         </is>
       </c>
-      <c r="C7" s="37" t="inlineStr">
+      <c r="C19" s="37" t="inlineStr">
         <is>
           <t>Apr 1-14</t>
         </is>
       </c>
-      <c r="D7" s="38" t="inlineStr">
+      <c r="D19" s="38" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="E7" s="39" t="inlineStr">
+      <c r="E19" s="39" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F7" s="40" t="inlineStr">
+      <c r="F19" s="40" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="G7" s="41" t="inlineStr">
+      <c r="G19" s="41" t="inlineStr">
         <is>
           <t>Deliverables from Quannex/Phase 2</t>
         </is>
       </c>
-      <c r="H7" s="36" t="inlineStr">
-        <is>
-          <t>Both questionnaires returned Apr 7. 14-doc evidence package. BSC 5/6. FOLDER EMPTY</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="H19" s="36" t="inlineStr">
+        <is>
+          <t>Both questionnaires Apr 7. 14-doc evidence package. BSC 5/6. FOLDER EMPTY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
         <is>
           <t>Phase 3</t>
         </is>
       </c>
-      <c r="B8" s="36" t="inlineStr">
-        <is>
-          <t>Validation session with D + E</t>
-        </is>
-      </c>
-      <c r="C8" s="37" t="inlineStr">
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>Results presentation + validation + debrief</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
         <is>
           <t>Apr 15-30</t>
         </is>
       </c>
-      <c r="D8" s="42" t="inlineStr">
+      <c r="D20" s="53" t="inlineStr">
         <is>
           <t>UPCOMING</t>
         </is>
       </c>
-      <c r="E8" s="43" t="inlineStr">
+      <c r="E20" s="54" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="F20" s="40" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F8" s="43" t="inlineStr">
+      <c r="G20" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables from Quannex/Phase 3</t>
+        </is>
+      </c>
+      <c r="H20" s="36" t="inlineStr">
+        <is>
+          <t>~April 17. Need: presentation, CEN summary, 3D demo (needs CEN template).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B21" s="36" t="inlineStr">
+        <is>
+          <t>Final report + KPIs + acknowledgment</t>
+        </is>
+      </c>
+      <c r="C21" s="37" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="D21" s="55" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="E21" s="43" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="G8" s="41" t="inlineStr">
-        <is>
-          <t>Deliverables from Quannex/Phase 3</t>
-        </is>
-      </c>
-      <c r="H8" s="36" t="inlineStr">
-        <is>
-          <t>Present coherence portrait. ~Apr 17. Prepare CEN-facing summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="35" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="inlineStr">
-        <is>
-          <t>Final report + recommendations</t>
-        </is>
-      </c>
-      <c r="C9" s="37" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D9" s="43" t="inlineStr">
+      <c r="F21" s="37" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G21" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables from Quannex/Phase 4</t>
+        </is>
+      </c>
+      <c r="H21" s="36" t="inlineStr">
+        <is>
+          <t>Depends on Phase 3 validation + thesis chapters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>PACKAGING ACTIONS — What needs to happen before Phase 3 (~April 17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="44" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B24" s="44" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C24" s="44" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D24" s="44" t="inlineStr">
+        <is>
+          <t>Output Format</t>
+        </is>
+      </c>
+      <c r="E24" s="44" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+      <c r="F24" s="44" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G24" s="44" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="H24" s="44" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="40" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="B25" s="45" t="inlineStr">
+        <is>
+          <t>Create CEN company template for POC</t>
+        </is>
+      </c>
+      <c r="C25" s="36" t="inlineStr">
+        <is>
+          <t>RawScores_Frozen.md (normalized arrays ready)</t>
+        </is>
+      </c>
+      <c r="D25" s="36" t="inlineStr">
+        <is>
+          <t>companies/cen/ (company.json + kpis.csv + mapping-context.json)</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="inlineStr">
+        <is>
+          <t>POC/companies/cen/</t>
+        </is>
+      </c>
+      <c r="F25" s="37" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+      <c r="G25" s="37" t="inlineStr">
+        <is>
+          <t>~2 hours</t>
+        </is>
+      </c>
+      <c r="H25" s="36" t="inlineStr">
+        <is>
+          <t>Unlocks: 3D visualization (#3), shadow analysis (#4), live demo. D_norm + E_norm available. Use average or researcher-calibrated vector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="B26" s="45" t="inlineStr">
+        <is>
+          <t>Create Phase 3 validation presentation</t>
+        </is>
+      </c>
+      <c r="C26" s="36" t="inlineStr">
+        <is>
+          <t>Phase 2 evidence package (C1-C4 docs)</t>
+        </is>
+      </c>
+      <c r="D26" s="36" t="inlineStr">
+        <is>
+          <t>PPTX (Quannex branded)</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables/Phase 3/</t>
+        </is>
+      </c>
+      <c r="F26" s="37" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+      <c r="G26" s="37" t="inlineStr">
+        <is>
+          <t>~3 hours</t>
+        </is>
+      </c>
+      <c r="H26" s="36" t="inlineStr">
+        <is>
+          <t>The centerpiece of the ~April 17 meeting. Coherence portrait + key findings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="40" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="B27" s="45" t="inlineStr">
+        <is>
+          <t>Create CEN-facing coherence summary</t>
+        </is>
+      </c>
+      <c r="C27" s="36" t="inlineStr">
+        <is>
+          <t>C1 Vector Diagnostics + C2 Breath + C3 Divergence</t>
+        </is>
+      </c>
+      <c r="D27" s="36" t="inlineStr">
+        <is>
+          <t>PDF (Quannex branded, 2-4 pages)</t>
+        </is>
+      </c>
+      <c r="E27" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables/Phase 3/</t>
+        </is>
+      </c>
+      <c r="F27" s="37" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+      <c r="G27" s="37" t="inlineStr">
+        <is>
+          <t>~2 hours</t>
+        </is>
+      </c>
+      <c r="H27" s="36" t="inlineStr">
+        <is>
+          <t>Executive summary leave-behind document for D and E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B28" s="45" t="inlineStr">
+        <is>
+          <t>Package Phase 1 deliverables</t>
+        </is>
+      </c>
+      <c r="C28" s="36" t="inlineStr">
+        <is>
+          <t>Interview synthesis (57KB) + face mapping (33KB)</t>
+        </is>
+      </c>
+      <c r="D28" s="36" t="inlineStr">
+        <is>
+          <t>PDF (Quannex branded)</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables/Phase 1/</t>
+        </is>
+      </c>
+      <c r="F28" s="37" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+      <c r="G28" s="37" t="inlineStr">
+        <is>
+          <t>~1 hour</t>
+        </is>
+      </c>
+      <c r="H28" s="36" t="inlineStr">
+        <is>
+          <t>Overdue (was due late March). Format existing MDs to branded PDFs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B29" s="45" t="inlineStr">
+        <is>
+          <t>Package Phase 2 deliverables</t>
+        </is>
+      </c>
+      <c r="C29" s="36" t="inlineStr">
+        <is>
+          <t>Evidence package C1-C4 + BSC comparison + breath analysis</t>
+        </is>
+      </c>
+      <c r="D29" s="36" t="inlineStr">
+        <is>
+          <t>PDF (Quannex branded)</t>
+        </is>
+      </c>
+      <c r="E29" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables/Phase 2/</t>
+        </is>
+      </c>
+      <c r="F29" s="37" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+      <c r="G29" s="37" t="inlineStr">
+        <is>
+          <t>~2 hours</t>
+        </is>
+      </c>
+      <c r="H29" s="36" t="inlineStr">
+        <is>
+          <t>Overdue (was due early April). Format existing MDs to branded PDFs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B30" s="45" t="inlineStr">
+        <is>
+          <t>Package conventional analysis</t>
+        </is>
+      </c>
+      <c r="C30" s="36" t="inlineStr">
+        <is>
+          <t>CEN_Conventional_Analysis_Working_Draft.md (77KB)</t>
+        </is>
+      </c>
+      <c r="D30" s="36" t="inlineStr">
+        <is>
+          <t>PDF (Quannex branded)</t>
+        </is>
+      </c>
+      <c r="E30" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables/Phase 1/ or Phase 2/</t>
+        </is>
+      </c>
+      <c r="F30" s="37" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+      <c r="G30" s="37" t="inlineStr">
+        <is>
+          <t>~1 hour</t>
+        </is>
+      </c>
+      <c r="H30" s="36" t="inlineStr">
+        <is>
+          <t>Promised deliverable #1. PESTEL + 7S + SWOT + BSC. Post-interview enriched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="43" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="B31" s="45" t="inlineStr">
+        <is>
+          <t>Prepare KPI proposals</t>
+        </is>
+      </c>
+      <c r="C31" s="36" t="inlineStr">
+        <is>
+          <t>Derive from coherence portrait + face mapping</t>
+        </is>
+      </c>
+      <c r="D31" s="36" t="inlineStr">
+        <is>
+          <t>PDF or section in final report</t>
+        </is>
+      </c>
+      <c r="E31" s="41" t="inlineStr">
+        <is>
+          <t>Deliverables/Phase 3/ or Phase 4/</t>
+        </is>
+      </c>
+      <c r="F31" s="37" t="inlineStr">
         <is>
           <t>NOT STARTED</t>
         </is>
       </c>
-      <c r="E9" s="43" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F9" s="43" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G9" s="41" t="inlineStr">
-        <is>
-          <t>Deliverables from Quannex/Phase 4</t>
-        </is>
-      </c>
-      <c r="H9" s="36" t="inlineStr">
-        <is>
-          <t>Depends on Ch5 + cross-case analysis completion</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>PHASE 1 DELIVERABLES — Package into: Deliverables from Quannex/Phase 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="44" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
-        </is>
-      </c>
-      <c r="B12" s="44" t="inlineStr">
-        <is>
-          <t>Source Material</t>
-        </is>
-      </c>
-      <c r="C12" s="44" t="inlineStr">
-        <is>
-          <t>Source Location</t>
-        </is>
-      </c>
-      <c r="D12" s="44" t="inlineStr">
-        <is>
-          <t>Format</t>
-        </is>
-      </c>
-      <c r="E12" s="44" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F12" s="44" t="inlineStr">
-        <is>
-          <t>Action Needed</t>
-        </is>
-      </c>
-      <c r="G12" s="44" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H12" s="44" t="inlineStr">
+      <c r="G31" s="37" t="inlineStr">
+        <is>
+          <t>~2 hours</t>
+        </is>
+      </c>
+      <c r="H31" s="36" t="inlineStr">
+        <is>
+          <t>Promised deliverable #7. Can be preliminary for Phase 3, finalized Phase 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="43" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B32" s="45" t="inlineStr">
+        <is>
+          <t>Run CEN data through POC engine</t>
+        </is>
+      </c>
+      <c r="C32" s="36" t="inlineStr">
+        <is>
+          <t>CEN company template (after creation)</t>
+        </is>
+      </c>
+      <c r="D32" s="36" t="inlineStr">
+        <is>
+          <t>Screenshots + engine output for presentation</t>
+        </is>
+      </c>
+      <c r="E32" s="41" t="inlineStr">
+        <is>
+          <t>Phase 3 presentation</t>
+        </is>
+      </c>
+      <c r="F32" s="37" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G32" s="37" t="inlineStr">
+        <is>
+          <t>~30 min</t>
+        </is>
+      </c>
+      <c r="H32" s="36" t="inlineStr">
+        <is>
+          <t>Blocked on CEN template creation. Once created, engine runs automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="33" t="inlineStr">
+        <is>
+          <t>CEN RAW SCORES (frozen Apr 8 — from RawScores_Frozen.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="44" t="inlineStr">
+        <is>
+          <t>Face</t>
+        </is>
+      </c>
+      <c r="B35" s="44" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="C35" s="44" t="inlineStr">
+        <is>
+          <t>D (Dominique)</t>
+        </is>
+      </c>
+      <c r="D35" s="44" t="inlineStr">
+        <is>
+          <t>E (Esther)</t>
+        </is>
+      </c>
+      <c r="E35" s="44" t="inlineStr">
+        <is>
+          <t>V_res_post</t>
+        </is>
+      </c>
+      <c r="F35" s="44" t="inlineStr">
+        <is>
+          <t>|D-E|</t>
+        </is>
+      </c>
+      <c r="G35" s="44" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="H35" s="44" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="45" t="inlineStr">
-        <is>
-          <t>Interview Synthesis Report</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="inlineStr">
-        <is>
-          <t>CEN_Phase1_Interview_Synthesis.md (57 KB)</t>
-        </is>
-      </c>
-      <c r="C13" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase1/</t>
-        </is>
-      </c>
-      <c r="D13" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E13" s="46" t="inlineStr">
-        <is>
-          <t>EXISTS — needs formatting</t>
-        </is>
-      </c>
-      <c r="F13" s="36" t="inlineStr">
-        <is>
-          <t>Convert to branded PDF, add exec summary</t>
-        </is>
-      </c>
-      <c r="G13" s="47" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B36" s="36" t="inlineStr">
+        <is>
+          <t>Financial Capital</t>
+        </is>
+      </c>
+      <c r="C36" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="G36" s="49" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="H13" s="36" t="inlineStr">
-        <is>
-          <t>Core research artifact — shows CEN their organizational portrait from Phase 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="45" t="inlineStr">
-        <is>
-          <t>Preliminary Face Mapping</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="inlineStr">
-        <is>
-          <t>CEN_Preliminary_Face_Mapping.md (33 KB)</t>
-        </is>
-      </c>
-      <c r="C14" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase1/</t>
-        </is>
-      </c>
-      <c r="D14" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E14" s="46" t="inlineStr">
-        <is>
-          <t>EXISTS — needs formatting</t>
-        </is>
-      </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>Convert to branded PDF with visual dodecahedron diagram</t>
-        </is>
-      </c>
-      <c r="G14" s="47" t="inlineStr">
+      <c r="H36" s="36" t="inlineStr">
+        <is>
+          <t>Biggest co-founder gap after F8</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B37" s="36" t="inlineStr">
+        <is>
+          <t>Intellectual Capital</t>
+        </is>
+      </c>
+      <c r="C37" s="37" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="E37" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="37" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="H37" s="36" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="35" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B38" s="36" t="inlineStr">
+        <is>
+          <t>Human Capital</t>
+        </is>
+      </c>
+      <c r="C38" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="D38" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="F38" s="54" t="n">
+        <v>4</v>
+      </c>
+      <c r="G38" s="49" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="H14" s="36" t="inlineStr">
-        <is>
-          <t>Shows how CEN's domains map to the 12 faces</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="45" t="inlineStr">
-        <is>
-          <t>Meeting Transcript</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="inlineStr">
-        <is>
-          <t>20-03-2026_PHASE1_Meeting-TRANSCRIPT.md (183 KB)</t>
-        </is>
-      </c>
-      <c r="C15" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase1/</t>
-        </is>
-      </c>
-      <c r="D15" s="37" t="inlineStr">
-        <is>
-          <t>PDF or MD</t>
-        </is>
-      </c>
-      <c r="E15" s="48" t="inlineStr">
-        <is>
-          <t>EXISTS — decide if CEN-facing</t>
-        </is>
-      </c>
-      <c r="F15" s="36" t="inlineStr">
-        <is>
-          <t>Review for sensitivity, redact if needed</t>
-        </is>
-      </c>
-      <c r="G15" s="49" t="inlineStr">
+      <c r="H38" s="36" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>Structural Capital</t>
+        </is>
+      </c>
+      <c r="C39" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="D39" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="G39" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H39" s="36" t="inlineStr">
+        <is>
+          <t>2-vs-1 pattern: E=V_res=2, D=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="35" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B40" s="36" t="inlineStr">
+        <is>
+          <t>Market Resonance</t>
+        </is>
+      </c>
+      <c r="C40" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" s="37" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="H15" s="36" t="inlineStr">
-        <is>
-          <t>May not need to be delivered — check partnership agreement</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="45" t="inlineStr">
-        <is>
-          <t>Personal Notes</t>
-        </is>
-      </c>
-      <c r="B16" s="36" t="inlineStr">
-        <is>
-          <t>Personal Notes - Fresh, right after the meeting!.md</t>
-        </is>
-      </c>
-      <c r="C16" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase1/</t>
-        </is>
-      </c>
-      <c r="D16" s="37" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E16" s="48" t="inlineStr">
-        <is>
-          <t>INTERNAL ONLY</t>
-        </is>
-      </c>
-      <c r="F16" s="36" t="inlineStr">
-        <is>
-          <t>Do NOT deliver — keep as research evidence</t>
-        </is>
-      </c>
-      <c r="G16" s="37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="36" t="inlineStr">
-        <is>
-          <t>Raw observations, thesis evidence only</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="33" t="inlineStr">
-        <is>
-          <t>PHASE 2 DELIVERABLES — Package into: Deliverables from Quannex/Phase 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="44" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
-        </is>
-      </c>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t>Source Material</t>
-        </is>
-      </c>
-      <c r="C19" s="44" t="inlineStr">
-        <is>
-          <t>Source Location</t>
-        </is>
-      </c>
-      <c r="D19" s="44" t="inlineStr">
-        <is>
-          <t>Format</t>
-        </is>
-      </c>
-      <c r="E19" s="44" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F19" s="44" t="inlineStr">
-        <is>
-          <t>Action Needed</t>
-        </is>
-      </c>
-      <c r="G19" s="44" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H19" s="44" t="inlineStr">
+      <c r="H40" s="36" t="inlineStr">
+        <is>
+          <t>Both low</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="35" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="B41" s="36" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C41" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="37" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="H41" s="36" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="35" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="B42" s="36" t="inlineStr">
+        <is>
+          <t>Brand &amp; Reputation</t>
+        </is>
+      </c>
+      <c r="C42" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="D42" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="54" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H42" s="36" t="inlineStr">
+        <is>
+          <t>2-vs-1 pattern: E=V_res=3, D=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="B43" s="36" t="inlineStr">
+        <is>
+          <t>Core Operations</t>
+        </is>
+      </c>
+      <c r="C43" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="D43" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" s="56" t="n">
+        <v>6</v>
+      </c>
+      <c r="G43" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="H43" s="36" t="inlineStr">
+        <is>
+          <t>Largest gap. 2-vs-1 pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="35" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="B44" s="36" t="inlineStr">
+        <is>
+          <t>Regenerative Flow</t>
+        </is>
+      </c>
+      <c r="C44" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="D44" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E44" s="37" t="n">
+        <v>8</v>
+      </c>
+      <c r="F44" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="37" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="H44" s="36" t="inlineStr">
+        <is>
+          <t>Researcher sees this highest</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="35" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B45" s="36" t="inlineStr">
+        <is>
+          <t>Foundational Values</t>
+        </is>
+      </c>
+      <c r="C45" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="37" t="n">
+        <v>9</v>
+      </c>
+      <c r="E45" s="37" t="n">
+        <v>8</v>
+      </c>
+      <c r="F45" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="37" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="H45" s="36" t="inlineStr">
+        <is>
+          <t>Consensus strength</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="B46" s="36" t="inlineStr">
+        <is>
+          <t>Funding Pipeline</t>
+        </is>
+      </c>
+      <c r="C46" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="D46" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="G46" s="37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="H46" s="36" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="35" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="B47" s="36" t="inlineStr">
+        <is>
+          <t>Risk &amp; Resilience</t>
+        </is>
+      </c>
+      <c r="C47" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D47" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" s="37" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="H47" s="36" t="inlineStr">
+        <is>
+          <t>Both co-founders see weakness</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="45" t="inlineStr"/>
+      <c r="B48" s="45" t="inlineStr">
+        <is>
+          <t>Overall Coherence</t>
+        </is>
+      </c>
+      <c r="C48" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="D48" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="37" t="inlineStr"/>
+      <c r="F48" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="G48" s="49" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H48" s="36" t="inlineStr">
+        <is>
+          <t>Macro gap matches micro face-level gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="41" t="inlineStr">
+        <is>
+          <t>POC-READY NORMALIZED ARRAYS (from RawScores_Frozen.md — paste into companies/cen/kpis.csv)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="41" t="inlineStr">
+        <is>
+          <t>D_norm = [0.6, 0.8, 0.7, 0.7, 0.3, 0.3, 0.7, 0.7, 0.6, 1.0, 0.6, 0.3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>E_norm = [0.1, 0.7, 0.3, 0.2, 0.1, 0.4, 0.3, 0.1, 0.5, 0.9, 0.4, 0.1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="41" t="inlineStr">
+        <is>
+          <t>V_res_post_norm = [0.2, 0.5, 0.4, 0.2, 0.2, 0.4, 0.3, 0.2, 0.8, 0.8, 0.2, 0.3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="33" t="inlineStr">
+        <is>
+          <t>CEN INPUT MATERIALS RECEIVED (reference inventory)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="44" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B56" s="44" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C56" s="44" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="D56" s="44" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="E56" s="44" t="inlineStr">
+        <is>
+          <t>Relevance</t>
+        </is>
+      </c>
+      <c r="F56" s="44" t="inlineStr">
+        <is>
+          <t>Used In</t>
+        </is>
+      </c>
+      <c r="G56" s="44" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="45" t="inlineStr">
-        <is>
-          <t>Coherence Portrait / Vector Diagnostics</t>
-        </is>
-      </c>
-      <c r="B20" s="36" t="inlineStr">
-        <is>
-          <t>CEN_Phase2_C1_VectorDiagnostics.md (20 KB)</t>
-        </is>
-      </c>
-      <c r="C20" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
-        </is>
-      </c>
-      <c r="D20" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E20" s="46" t="inlineStr">
-        <is>
-          <t>EXISTS — needs formatting</t>
-        </is>
-      </c>
-      <c r="F20" s="36" t="inlineStr">
-        <is>
-          <t>Convert to branded CEN-facing report, add visualizations</t>
-        </is>
-      </c>
-      <c r="G20" s="47" t="inlineStr">
+      <c r="H56" s="44" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="36" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="B57" s="45" t="inlineStr">
+        <is>
+          <t>Signed NDA</t>
+        </is>
+      </c>
+      <c r="C57" s="37" t="inlineStr">
+        <is>
+          <t>461 KB</t>
+        </is>
+      </c>
+      <c r="D57" s="41" t="inlineStr">
+        <is>
+          <t>Meeting 1st/</t>
+        </is>
+      </c>
+      <c r="E57" s="37" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F57" s="36" t="inlineStr">
+        <is>
+          <t>All phases</t>
+        </is>
+      </c>
+      <c r="G57" s="36" t="inlineStr">
+        <is>
+          <t>Feb 15, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="36" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="B58" s="45" t="inlineStr">
+        <is>
+          <t>Signed Partnership Confirmation</t>
+        </is>
+      </c>
+      <c r="C58" s="37" t="inlineStr">
+        <is>
+          <t>409 KB</t>
+        </is>
+      </c>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>Meeting 1st/</t>
+        </is>
+      </c>
+      <c r="E58" s="37" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F58" s="36" t="inlineStr">
+        <is>
+          <t>All phases</t>
+        </is>
+      </c>
+      <c r="G58" s="36" t="inlineStr">
+        <is>
+          <t>Feb 15, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="36" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B59" s="45" t="inlineStr">
+        <is>
+          <t>CEN Business Plan V2.0</t>
+        </is>
+      </c>
+      <c r="C59" s="37" t="inlineStr">
+        <is>
+          <t>~19 MB</t>
+        </is>
+      </c>
+      <c r="D59" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Strategy/</t>
+        </is>
+      </c>
+      <c r="E59" s="49" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="H20" s="36" t="inlineStr">
-        <is>
-          <t>The core deliverable — shows CEN their coherence state</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="45" t="inlineStr">
-        <is>
-          <t>Breath Axis Analysis</t>
-        </is>
-      </c>
-      <c r="B21" s="36" t="inlineStr">
-        <is>
-          <t>CEN_Phase2_C2_BreathAxes.md (21 KB)</t>
-        </is>
-      </c>
-      <c r="C21" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
-        </is>
-      </c>
-      <c r="D21" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E21" s="46" t="inlineStr">
-        <is>
-          <t>EXISTS — needs formatting</t>
-        </is>
-      </c>
-      <c r="F21" s="36" t="inlineStr">
-        <is>
-          <t>Format as section of coherence report or standalone</t>
-        </is>
-      </c>
-      <c r="G21" s="47" t="inlineStr">
+      <c r="F59" s="36" t="inlineStr">
+        <is>
+          <t>Phase 1 synthesis</t>
+        </is>
+      </c>
+      <c r="G59" s="36" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="36" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B60" s="45" t="inlineStr">
+        <is>
+          <t>CEN Strategy V0.4</t>
+        </is>
+      </c>
+      <c r="C60" s="37" t="inlineStr">
+        <is>
+          <t>425 KB</t>
+        </is>
+      </c>
+      <c r="D60" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Strategy/</t>
+        </is>
+      </c>
+      <c r="E60" s="49" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="H21" s="36" t="inlineStr">
-        <is>
-          <t>Polarity tensions — key insight for leadership</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="45" t="inlineStr">
-        <is>
-          <t>Divergence Narratives (Hidden Tensions)</t>
-        </is>
-      </c>
-      <c r="B22" s="36" t="inlineStr">
-        <is>
-          <t>CEN_Phase2_C3_DivergenceNarratives.md (13 KB)</t>
-        </is>
-      </c>
-      <c r="C22" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
-        </is>
-      </c>
-      <c r="D22" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E22" s="46" t="inlineStr">
-        <is>
-          <t>EXISTS — needs formatting</t>
-        </is>
-      </c>
-      <c r="F22" s="36" t="inlineStr">
-        <is>
-          <t>Sensitive content — frame constructively for CEN</t>
-        </is>
-      </c>
-      <c r="G22" s="47" t="inlineStr">
+      <c r="F60" s="36" t="inlineStr">
+        <is>
+          <t>Phase 1 synthesis</t>
+        </is>
+      </c>
+      <c r="G60" s="36" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="36" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B61" s="45" t="inlineStr">
+        <is>
+          <t>Purpose Vision Mission Values V0.1</t>
+        </is>
+      </c>
+      <c r="C61" s="37" t="inlineStr">
+        <is>
+          <t>25 KB</t>
+        </is>
+      </c>
+      <c r="D61" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Vision Mission/</t>
+        </is>
+      </c>
+      <c r="E61" s="49" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="H22" s="36" t="inlineStr">
-        <is>
-          <t>Where co-founders diverge — handle with care</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="45" t="inlineStr">
-        <is>
-          <t>BSC Comparison Report</t>
-        </is>
-      </c>
-      <c r="B23" s="36" t="inlineStr">
-        <is>
-          <t>CEN_Phase2_C4_BSCComparison.md (27 KB)</t>
-        </is>
-      </c>
-      <c r="C23" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
-        </is>
-      </c>
-      <c r="D23" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E23" s="46" t="inlineStr">
-        <is>
-          <t>EXISTS — needs formatting</t>
-        </is>
-      </c>
-      <c r="F23" s="36" t="inlineStr">
-        <is>
-          <t>Format as comparison report: Spiral vs BSC (5/6 verdict)</t>
-        </is>
-      </c>
-      <c r="G23" s="47" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="H23" s="36" t="inlineStr">
-        <is>
-          <t>Academic evidence + CEN value prop: shows what Spiral adds over BSC</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="45" t="inlineStr">
-        <is>
-          <t>Raw Scoring Data (Frozen)</t>
-        </is>
-      </c>
-      <c r="B24" s="36" t="inlineStr">
-        <is>
-          <t>CEN_Phase2_RawScores_Frozen.md (9 KB)</t>
-        </is>
-      </c>
-      <c r="C24" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase2/EvidencePackage/</t>
-        </is>
-      </c>
-      <c r="D24" s="37" t="inlineStr">
-        <is>
-          <t>PDF or Excel</t>
-        </is>
-      </c>
-      <c r="E24" s="48" t="inlineStr">
-        <is>
-          <t>EXISTS — decide if CEN-facing</t>
-        </is>
-      </c>
-      <c r="F24" s="36" t="inlineStr">
-        <is>
-          <t>May include as appendix to coherence portrait</t>
-        </is>
-      </c>
-      <c r="G24" s="49" t="inlineStr">
+      <c r="F61" s="36" t="inlineStr">
+        <is>
+          <t>Face mapping</t>
+        </is>
+      </c>
+      <c r="G61" s="36" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="36" t="inlineStr">
+        <is>
+          <t>Pillar 1-3</t>
+        </is>
+      </c>
+      <c r="B62" s="45" t="inlineStr">
+        <is>
+          <t>CEN organizational documents (28 files)</t>
+        </is>
+      </c>
+      <c r="C62" s="37" t="inlineStr">
+        <is>
+          <t>~44 MB</t>
+        </is>
+      </c>
+      <c r="D62" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Documents &amp; Policies/</t>
+        </is>
+      </c>
+      <c r="E62" s="37" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="H24" s="36" t="inlineStr">
-        <is>
-          <t>Both co-founders' scores, independence verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="45" t="inlineStr">
-        <is>
-          <t>Scoring Questionnaires (Completed)</t>
-        </is>
-      </c>
-      <c r="B25" s="36" t="inlineStr">
-        <is>
-          <t>Dominique + Esther completed questionnaires</t>
-        </is>
-      </c>
-      <c r="C25" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/CEN_Scoring_Questionnaire/</t>
-        </is>
-      </c>
-      <c r="D25" s="37" t="inlineStr">
-        <is>
-          <t>DOCX (as-is)</t>
-        </is>
-      </c>
-      <c r="E25" s="50" t="inlineStr">
-        <is>
-          <t>COMPLETE — already received</t>
-        </is>
-      </c>
-      <c r="F25" s="36" t="inlineStr">
-        <is>
-          <t>Archive copies in Phase 2 folder for completeness</t>
-        </is>
-      </c>
-      <c r="G25" s="37" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="H25" s="36" t="inlineStr">
-        <is>
-          <t>Input FROM CEN, not deliverable TO CEN — but archive</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="45" t="inlineStr">
-        <is>
-          <t>Face Guide Companion</t>
-        </is>
-      </c>
-      <c r="B26" s="36" t="inlineStr">
-        <is>
-          <t>CEN_Face_Guide_For_Scoring.pdf (202 KB)</t>
-        </is>
-      </c>
-      <c r="C26" s="41" t="inlineStr">
-        <is>
-          <t>Meetings &amp; Planning/CEN_Phase2/</t>
-        </is>
-      </c>
-      <c r="D26" s="37" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="E26" s="50" t="inlineStr">
-        <is>
-          <t>COMPLETE</t>
-        </is>
-      </c>
-      <c r="F26" s="36" t="inlineStr">
-        <is>
-          <t>Already formatted — copy to Phase 2 folder</t>
-        </is>
-      </c>
-      <c r="G26" s="37" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="H26" s="36" t="inlineStr">
-        <is>
-          <t>Sent to CEN for scoring context</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="33" t="inlineStr">
-        <is>
-          <t>PHASE 3 DELIVERABLES — Validation Session (~April 17) — Package into: Deliverables from Quannex/Phase 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="44" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
-        </is>
-      </c>
-      <c r="B29" s="44" t="inlineStr">
-        <is>
-          <t>Source Material</t>
-        </is>
-      </c>
-      <c r="C29" s="44" t="inlineStr">
-        <is>
-          <t>Source Location</t>
-        </is>
-      </c>
-      <c r="D29" s="44" t="inlineStr">
-        <is>
-          <t>Format</t>
-        </is>
-      </c>
-      <c r="E29" s="44" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F29" s="44" t="inlineStr">
-        <is>
-          <t>Action Needed</t>
-        </is>
-      </c>
-      <c r="G29" s="44" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H29" s="44" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="45" t="inlineStr">
-        <is>
-          <t>Validation Presentation</t>
-        </is>
-      </c>
-      <c r="B30" s="36" t="inlineStr">
-        <is>
-          <t>To be created from Phase 2 evidence</t>
-        </is>
-      </c>
-      <c r="C30" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D30" s="37" t="inlineStr">
-        <is>
-          <t>PPTX (branded)</t>
-        </is>
-      </c>
-      <c r="E30" s="51" t="inlineStr">
-        <is>
-          <t>NOT STARTED</t>
-        </is>
-      </c>
-      <c r="F30" s="36" t="inlineStr">
-        <is>
-          <t>Create presentation summarizing coherence portrait + key findings</t>
-        </is>
-      </c>
-      <c r="G30" s="47" t="inlineStr">
+      <c r="F62" s="36" t="inlineStr">
+        <is>
+          <t>Conventional analysis</t>
+        </is>
+      </c>
+      <c r="G62" s="36" t="inlineStr">
+        <is>
+          <t>Education, AI, LLM, Business Plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="36" t="inlineStr">
+        <is>
+          <t>Scoring</t>
+        </is>
+      </c>
+      <c r="B63" s="45" t="inlineStr">
+        <is>
+          <t>Dominique questionnaire (completed)</t>
+        </is>
+      </c>
+      <c r="C63" s="37" t="inlineStr">
+        <is>
+          <t>27 KB</t>
+        </is>
+      </c>
+      <c r="D63" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Scoring/</t>
+        </is>
+      </c>
+      <c r="E63" s="47" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="H30" s="36" t="inlineStr">
-        <is>
-          <t>This is what you present to D + E at the validation meeting</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="45" t="inlineStr">
-        <is>
-          <t>CEN-Facing Coherence Summary</t>
-        </is>
-      </c>
-      <c r="B31" s="36" t="inlineStr">
-        <is>
-          <t>Synthesize from C1-C4 evidence docs</t>
-        </is>
-      </c>
-      <c r="C31" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D31" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E31" s="51" t="inlineStr">
-        <is>
-          <t>NOT STARTED</t>
-        </is>
-      </c>
-      <c r="F31" s="36" t="inlineStr">
-        <is>
-          <t>One-page or two-page executive summary for CEN leadership</t>
-        </is>
-      </c>
-      <c r="G31" s="47" t="inlineStr">
+      <c r="F63" s="36" t="inlineStr">
+        <is>
+          <t>Phase 2 evidence</t>
+        </is>
+      </c>
+      <c r="G63" s="36" t="inlineStr">
+        <is>
+          <t>Returned Apr 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="36" t="inlineStr">
+        <is>
+          <t>Scoring</t>
+        </is>
+      </c>
+      <c r="B64" s="45" t="inlineStr">
+        <is>
+          <t>Esther questionnaire (completed)</t>
+        </is>
+      </c>
+      <c r="C64" s="37" t="inlineStr">
+        <is>
+          <t>30 KB</t>
+        </is>
+      </c>
+      <c r="D64" s="41" t="inlineStr">
+        <is>
+          <t>CEN Inputs/Scoring/</t>
+        </is>
+      </c>
+      <c r="E64" s="47" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="H31" s="36" t="inlineStr">
-        <is>
-          <t>Leave-behind document after validation session</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="45" t="inlineStr">
-        <is>
-          <t>Validation Session Notes</t>
-        </is>
-      </c>
-      <c r="B32" s="36" t="inlineStr">
-        <is>
-          <t>Will be captured during meeting</t>
-        </is>
-      </c>
-      <c r="C32" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D32" s="37" t="inlineStr">
-        <is>
-          <t>MD then PDF</t>
-        </is>
-      </c>
-      <c r="E32" s="48" t="inlineStr">
-        <is>
-          <t>FUTURE</t>
-        </is>
-      </c>
-      <c r="F32" s="36" t="inlineStr">
-        <is>
-          <t>Record CEN's reactions, corrections, confirmations</t>
-        </is>
-      </c>
-      <c r="G32" s="49" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="H32" s="36" t="inlineStr">
-        <is>
-          <t>Critical thesis evidence — did CEN validate the portrait?</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="45" t="inlineStr">
-        <is>
-          <t>POC Live Demo (optional)</t>
-        </is>
-      </c>
-      <c r="B33" s="36" t="inlineStr">
-        <is>
-          <t>POC codebase — load CEN data into engine</t>
-        </is>
-      </c>
-      <c r="C33" s="41" t="inlineStr">
-        <is>
-          <t>POC/companies/ (needs CEN template)</t>
-        </is>
-      </c>
-      <c r="D33" s="37" t="inlineStr">
-        <is>
-          <t>Live demo</t>
-        </is>
-      </c>
-      <c r="E33" s="48" t="inlineStr">
-        <is>
-          <t>REQUIRES CEN COMPANY TEMPLATE</t>
-        </is>
-      </c>
-      <c r="F33" s="36" t="inlineStr">
-        <is>
-          <t>Create companies/cen/ template from scoring data</t>
-        </is>
-      </c>
-      <c r="G33" s="49" t="inlineStr">
+      <c r="F64" s="36" t="inlineStr">
+        <is>
+          <t>Phase 2 evidence</t>
+        </is>
+      </c>
+      <c r="G64" s="36" t="inlineStr">
+        <is>
+          <t>Returned Apr 7. 3-4h investment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="36" t="inlineStr">
+        <is>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="B65" s="45" t="inlineStr">
+        <is>
+          <t>Phase 1 Interview (video)</t>
+        </is>
+      </c>
+      <c r="C65" s="37" t="inlineStr">
+        <is>
+          <t>4.08 GB</t>
+        </is>
+      </c>
+      <c r="D65" s="41" t="inlineStr">
+        <is>
+          <t>CEN_Phase1/</t>
+        </is>
+      </c>
+      <c r="E65" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="F65" s="36" t="inlineStr">
+        <is>
+          <t>Phase 1 synthesis</t>
+        </is>
+      </c>
+      <c r="G65" s="36" t="inlineStr">
+        <is>
+          <t>Mar 20, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="36" t="inlineStr">
+        <is>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="B66" s="45" t="inlineStr">
+        <is>
+          <t>Phase 2 Meeting (video)</t>
+        </is>
+      </c>
+      <c r="C66" s="37" t="inlineStr">
+        <is>
+          <t>430 MB</t>
+        </is>
+      </c>
+      <c r="D66" s="41" t="inlineStr">
+        <is>
+          <t>CEN_Phase2/</t>
+        </is>
+      </c>
+      <c r="E66" s="47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="F66" s="36" t="inlineStr">
+        <is>
+          <t>Phase 2 evidence</t>
+        </is>
+      </c>
+      <c r="G66" s="36" t="inlineStr">
+        <is>
+          <t>Apr 3, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="36" t="inlineStr">
+        <is>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="B67" s="45" t="inlineStr">
+        <is>
+          <t>Kick-Off meeting (video)</t>
+        </is>
+      </c>
+      <c r="C67" s="37" t="inlineStr">
+        <is>
+          <t>333 MB</t>
+        </is>
+      </c>
+      <c r="D67" s="41" t="inlineStr">
+        <is>
+          <t>Meeting 2nd/</t>
+        </is>
+      </c>
+      <c r="E67" s="37" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="H33" s="36" t="inlineStr">
-        <is>
-          <t>Would powerfully demonstrate the tool — consider creating CEN template from Phase 2 scores</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="33" t="inlineStr">
-        <is>
-          <t>PHASE 4 DELIVERABLES — Final Report (May) — Package into: Deliverables from Quannex/Phase 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="44" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
-        </is>
-      </c>
-      <c r="B36" s="44" t="inlineStr">
-        <is>
-          <t>Source Material</t>
-        </is>
-      </c>
-      <c r="C36" s="44" t="inlineStr">
-        <is>
-          <t>Source Location</t>
-        </is>
-      </c>
-      <c r="D36" s="44" t="inlineStr">
-        <is>
-          <t>Format</t>
-        </is>
-      </c>
-      <c r="E36" s="44" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F36" s="44" t="inlineStr">
-        <is>
-          <t>Action Needed</t>
-        </is>
-      </c>
-      <c r="G36" s="44" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H36" s="44" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="45" t="inlineStr">
-        <is>
-          <t>Final Coherence Report</t>
-        </is>
-      </c>
-      <c r="B37" s="36" t="inlineStr">
-        <is>
-          <t>Full synthesis of Phase 1-3 findings</t>
-        </is>
-      </c>
-      <c r="C37" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D37" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E37" s="48" t="inlineStr">
-        <is>
-          <t>NOT STARTED</t>
-        </is>
-      </c>
-      <c r="F37" s="36" t="inlineStr">
-        <is>
-          <t>Comprehensive CEN coherence assessment with recommendations</t>
-        </is>
-      </c>
-      <c r="G37" s="49" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="H37" s="36" t="inlineStr">
-        <is>
-          <t>The capstone deliverable — CEN's return on participation</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="45" t="inlineStr">
-        <is>
-          <t>Recommendations Document</t>
-        </is>
-      </c>
-      <c r="B38" s="36" t="inlineStr">
-        <is>
-          <t>Derived from cross-case analysis + validation</t>
-        </is>
-      </c>
-      <c r="C38" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D38" s="37" t="inlineStr">
-        <is>
-          <t>PDF (branded)</t>
-        </is>
-      </c>
-      <c r="E38" s="48" t="inlineStr">
-        <is>
-          <t>NOT STARTED</t>
-        </is>
-      </c>
-      <c r="F38" s="36" t="inlineStr">
-        <is>
-          <t>Actionable recommendations based on coherence portrait</t>
-        </is>
-      </c>
-      <c r="G38" s="49" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="H38" s="36" t="inlineStr">
-        <is>
-          <t>Practical value for CEN — not just academic</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="45" t="inlineStr">
-        <is>
-          <t>Thank You + Next Steps</t>
-        </is>
-      </c>
-      <c r="B39" s="36" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C39" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D39" s="37" t="inlineStr">
-        <is>
-          <t>PDF or letter</t>
-        </is>
-      </c>
-      <c r="E39" s="48" t="inlineStr">
-        <is>
-          <t>NOT STARTED</t>
-        </is>
-      </c>
-      <c r="F39" s="36" t="inlineStr">
-        <is>
-          <t>Formal closure of research partnership</t>
-        </is>
-      </c>
-      <c r="G39" s="37" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="H39" s="36" t="inlineStr">
-        <is>
-          <t>Professional courtesy — partnership confirmation referenced deliverables</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="33" t="inlineStr">
-        <is>
-          <t>CEN INPUT MATERIALS — Documents received from CEN (for reference)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="44" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B42" s="44" t="inlineStr">
-        <is>
-          <t>Document</t>
-        </is>
-      </c>
-      <c r="C42" s="44" t="inlineStr">
-        <is>
-          <t>Size</t>
-        </is>
-      </c>
-      <c r="D42" s="44" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="E42" s="44" t="inlineStr">
-        <is>
-          <t>Relevance</t>
-        </is>
-      </c>
-      <c r="F42" s="44" t="inlineStr">
-        <is>
-          <t>Used In</t>
-        </is>
-      </c>
-      <c r="G42" s="44" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="H42" s="44" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="36" t="inlineStr">
-        <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="B43" s="45" t="inlineStr">
-        <is>
-          <t>Signed NDA</t>
-        </is>
-      </c>
-      <c r="C43" s="37" t="inlineStr">
-        <is>
-          <t>461 KB</t>
-        </is>
-      </c>
-      <c r="D43" s="41" t="inlineStr">
-        <is>
-          <t>Meeting 1st/</t>
-        </is>
-      </c>
-      <c r="E43" s="37" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="F43" s="36" t="inlineStr">
-        <is>
-          <t>All phases</t>
-        </is>
-      </c>
-      <c r="G43" s="36" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="36" t="inlineStr">
-        <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="B44" s="45" t="inlineStr">
-        <is>
-          <t>Signed Partnership Confirmation</t>
-        </is>
-      </c>
-      <c r="C44" s="37" t="inlineStr">
-        <is>
-          <t>409 KB</t>
-        </is>
-      </c>
-      <c r="D44" s="41" t="inlineStr">
-        <is>
-          <t>Meeting 1st/</t>
-        </is>
-      </c>
-      <c r="E44" s="37" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="F44" s="36" t="inlineStr">
-        <is>
-          <t>All phases</t>
-        </is>
-      </c>
-      <c r="G44" s="36" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="36" t="inlineStr">
-        <is>
-          <t>Strategy</t>
-        </is>
-      </c>
-      <c r="B45" s="45" t="inlineStr">
-        <is>
-          <t>CEN Business Plan V2.0</t>
-        </is>
-      </c>
-      <c r="C45" s="37" t="inlineStr">
-        <is>
-          <t>~19 MB</t>
-        </is>
-      </c>
-      <c r="D45" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Strategy/</t>
-        </is>
-      </c>
-      <c r="E45" s="49" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="F45" s="36" t="inlineStr">
-        <is>
-          <t>Phase 1 synthesis</t>
-        </is>
-      </c>
-      <c r="G45" s="36" t="inlineStr">
-        <is>
-          <t>Core strategic context</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="36" t="inlineStr">
-        <is>
-          <t>Strategy</t>
-        </is>
-      </c>
-      <c r="B46" s="45" t="inlineStr">
-        <is>
-          <t>CEN Strategy V0.4</t>
-        </is>
-      </c>
-      <c r="C46" s="37" t="inlineStr">
-        <is>
-          <t>425 KB</t>
-        </is>
-      </c>
-      <c r="D46" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Strategy/</t>
-        </is>
-      </c>
-      <c r="E46" s="49" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="F46" s="36" t="inlineStr">
-        <is>
-          <t>Phase 1 synthesis</t>
-        </is>
-      </c>
-      <c r="G46" s="36" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="36" t="inlineStr">
-        <is>
-          <t>Strategy</t>
-        </is>
-      </c>
-      <c r="B47" s="45" t="inlineStr">
-        <is>
-          <t>Purpose Vision Mission Values V0.1</t>
-        </is>
-      </c>
-      <c r="C47" s="37" t="inlineStr">
-        <is>
-          <t>25 KB</t>
-        </is>
-      </c>
-      <c r="D47" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Vision Mission/</t>
-        </is>
-      </c>
-      <c r="E47" s="49" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="F47" s="36" t="inlineStr">
-        <is>
-          <t>Face mapping</t>
-        </is>
-      </c>
-      <c r="G47" s="36" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="36" t="inlineStr">
-        <is>
-          <t>Pillar 1</t>
-        </is>
-      </c>
-      <c r="B48" s="45" t="inlineStr">
-        <is>
-          <t>Conscious Leadership Course Proposal</t>
-        </is>
-      </c>
-      <c r="C48" s="37" t="inlineStr">
-        <is>
-          <t>1.2 MB</t>
-        </is>
-      </c>
-      <c r="D48" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Pillar 1/</t>
-        </is>
-      </c>
-      <c r="E48" s="37" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="F48" s="36" t="inlineStr">
-        <is>
-          <t>Face 6 (Consciousness)</t>
-        </is>
-      </c>
-      <c r="G48" s="36" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="36" t="inlineStr">
-        <is>
-          <t>Pillar 2</t>
-        </is>
-      </c>
-      <c r="B49" s="45" t="inlineStr">
-        <is>
-          <t>AI Consulting + Governance proposals</t>
-        </is>
-      </c>
-      <c r="C49" s="37" t="inlineStr">
-        <is>
-          <t>~230 KB</t>
-        </is>
-      </c>
-      <c r="D49" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Pillar 2/</t>
-        </is>
-      </c>
-      <c r="E49" s="37" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="F49" s="36" t="inlineStr">
-        <is>
-          <t>Face 3, Face 11</t>
-        </is>
-      </c>
-      <c r="G49" s="36" t="inlineStr">
-        <is>
-          <t>5 documents</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="36" t="inlineStr">
-        <is>
-          <t>Pillar 3</t>
-        </is>
-      </c>
-      <c r="B50" s="45" t="inlineStr">
-        <is>
-          <t>LLM, DCS, Business Plans, Partners</t>
-        </is>
-      </c>
-      <c r="C50" s="37" t="inlineStr">
-        <is>
-          <t>~42 MB</t>
-        </is>
-      </c>
-      <c r="D50" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Pillar 3/</t>
-        </is>
-      </c>
-      <c r="E50" s="37" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="F50" s="36" t="inlineStr">
-        <is>
-          <t>Multiple faces</t>
-        </is>
-      </c>
-      <c r="G50" s="36" t="inlineStr">
-        <is>
-          <t>18 documents</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="36" t="inlineStr">
-        <is>
-          <t>Teams</t>
-        </is>
-      </c>
-      <c r="B51" s="45" t="inlineStr">
-        <is>
-          <t>Volunteer programs + contracts</t>
-        </is>
-      </c>
-      <c r="C51" s="37" t="inlineStr">
-        <is>
-          <t>~470 KB</t>
-        </is>
-      </c>
-      <c r="D51" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Teams/</t>
-        </is>
-      </c>
-      <c r="E51" s="37" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="F51" s="36" t="inlineStr">
-        <is>
-          <t>Face 4, Face 9</t>
-        </is>
-      </c>
-      <c r="G51" s="36" t="inlineStr">
-        <is>
-          <t>5 documents</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="36" t="inlineStr">
-        <is>
-          <t>Scoring</t>
-        </is>
-      </c>
-      <c r="B52" s="45" t="inlineStr">
-        <is>
-          <t>Dominique questionnaire (completed)</t>
-        </is>
-      </c>
-      <c r="C52" s="37" t="inlineStr">
-        <is>
-          <t>27 KB</t>
-        </is>
-      </c>
-      <c r="D52" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Scoring/</t>
-        </is>
-      </c>
-      <c r="E52" s="47" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="F52" s="36" t="inlineStr">
-        <is>
-          <t>Phase 2 evidence</t>
-        </is>
-      </c>
-      <c r="G52" s="36" t="inlineStr">
-        <is>
-          <t>Returned Apr 7</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="36" t="inlineStr">
-        <is>
-          <t>Scoring</t>
-        </is>
-      </c>
-      <c r="B53" s="45" t="inlineStr">
-        <is>
-          <t>Esther questionnaire (completed)</t>
-        </is>
-      </c>
-      <c r="C53" s="37" t="inlineStr">
-        <is>
-          <t>30 KB</t>
-        </is>
-      </c>
-      <c r="D53" s="41" t="inlineStr">
-        <is>
-          <t>CEN Inputs/Scoring/</t>
-        </is>
-      </c>
-      <c r="E53" s="47" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="F53" s="36" t="inlineStr">
-        <is>
-          <t>Phase 2 evidence</t>
-        </is>
-      </c>
-      <c r="G53" s="36" t="inlineStr">
-        <is>
-          <t>Returned Apr 7</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="36" t="inlineStr">
-        <is>
-          <t>Recording</t>
-        </is>
-      </c>
-      <c r="B54" s="45" t="inlineStr">
-        <is>
-          <t>Phase 1 Interview (video)</t>
-        </is>
-      </c>
-      <c r="C54" s="37" t="inlineStr">
-        <is>
-          <t>4.08 GB</t>
-        </is>
-      </c>
-      <c r="D54" s="41" t="inlineStr">
-        <is>
-          <t>CEN_Phase1/</t>
-        </is>
-      </c>
-      <c r="E54" s="47" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="F54" s="36" t="inlineStr">
-        <is>
-          <t>Phase 1 synthesis</t>
-        </is>
-      </c>
-      <c r="G54" s="36" t="inlineStr">
-        <is>
-          <t>Primary research data</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="36" t="inlineStr">
-        <is>
-          <t>Recording</t>
-        </is>
-      </c>
-      <c r="B55" s="45" t="inlineStr">
-        <is>
-          <t>Phase 2 Meeting (video)</t>
-        </is>
-      </c>
-      <c r="C55" s="37" t="inlineStr">
-        <is>
-          <t>430 MB</t>
-        </is>
-      </c>
-      <c r="D55" s="41" t="inlineStr">
-        <is>
-          <t>CEN_Phase2/</t>
-        </is>
-      </c>
-      <c r="E55" s="47" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="F55" s="36" t="inlineStr">
-        <is>
-          <t>Phase 2 evidence</t>
-        </is>
-      </c>
-      <c r="G55" s="36" t="inlineStr">
-        <is>
-          <t>Primary research data</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="52" t="inlineStr">
-        <is>
-          <t>KEY GAP: Phase 1 and Phase 2 work is DONE but delivery folders are EMPTY. Package existing evidence into branded PDFs before Phase 3 validation (~April 17).</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="41" t="inlineStr">
-        <is>
-          <t>Folder path: Final Thesis/Thesis Work/External Partners/Coherence Partnership Quannex x CEN/Local Source for CEN facing documents/CEN Facing Folder/Deliverables from Quannex/</t>
+      <c r="F67" s="36" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="G67" s="36" t="inlineStr">
+        <is>
+          <t>Mar 13, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="52" t="inlineStr">
+        <is>
+          <t>KEY GAPS: (1) Delivery folders Phase 1-2 are EMPTY despite work being done. (2) CEN company template does not exist — blocks 3D viz, shadow analysis, live demo. (3) Proposed KPIs (#7) not started. (4) Conventional analysis exists but not CEN-facing.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A18:H18"/>
+  <mergeCells count="12">
+    <mergeCell ref="A50:H50"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A69:H69"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A52:H52"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation sqref="D6:D9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"DONE,UPCOMING,IN PROGRESS,NOT STARTED"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E6:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"YES,NO,PARTIAL"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>